<commit_message>
chore: update main pages
</commit_message>
<xml_diff>
--- a/CodeSystem-mii-cs-sdd-ausbildung.xlsx
+++ b/CodeSystem-mii-cs-sdd-ausbildung.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>2027.0.0-ballot.rc1</t>
+    <t>2027.0.0-ballot</t>
   </si>
   <si>
     <t>Name</t>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-09-14T13:12:23+00:00</t>
+    <t>2026-09-14T16:01:26+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>